<commit_message>
updated bulkdata file name to bulkdataxlsx
</commit_message>
<xml_diff>
--- a/src/test/resources/bulkDataXLSX.xlsx
+++ b/src/test/resources/bulkDataXLSX.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>Subhash</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>2024-08-23 08:23:30</t>
+  </si>
+  <si>
+    <t>2024-12-31 08:44:56</t>
   </si>
 </sst>
 </file>
@@ -453,7 +456,7 @@
         <v>85</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -473,7 +476,7 @@
         <v>63.89</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -493,7 +496,7 @@
         <v>70.56</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -513,7 +516,7 @@
         <v>80.010000000000005</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated config file paths
</commit_message>
<xml_diff>
--- a/src/test/resources/bulkDataXLSX.xlsx
+++ b/src/test/resources/bulkDataXLSX.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="27">
   <si>
     <t>Subhash</t>
   </si>
@@ -82,6 +82,30 @@
   </si>
   <si>
     <t>2024-12-31 08:44:56</t>
+  </si>
+  <si>
+    <t>2024-12-31 09:12:32</t>
+  </si>
+  <si>
+    <t>2024-12-31 09:15:19</t>
+  </si>
+  <si>
+    <t>2024-12-31 09:29:45</t>
+  </si>
+  <si>
+    <t>2024-12-31 09:37:23</t>
+  </si>
+  <si>
+    <t>2024-12-31 09:37:24</t>
+  </si>
+  <si>
+    <t>2024-12-31 10:12:49</t>
+  </si>
+  <si>
+    <t>2024-12-31 10:28:23</t>
+  </si>
+  <si>
+    <t>2024-12-31 10:52:39</t>
   </si>
 </sst>
 </file>
@@ -456,7 +480,7 @@
         <v>85</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -476,7 +500,7 @@
         <v>63.89</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -496,7 +520,7 @@
         <v>70.56</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -516,7 +540,7 @@
         <v>80.010000000000005</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
junit report added to plugin in test runner
</commit_message>
<xml_diff>
--- a/src/test/resources/bulkDataXLSX.xlsx
+++ b/src/test/resources/bulkDataXLSX.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="28">
   <si>
     <t>Subhash</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>2024-12-31 10:52:39</t>
+  </si>
+  <si>
+    <t>2025-01-01 07:27:49</t>
   </si>
 </sst>
 </file>
@@ -480,7 +483,7 @@
         <v>85</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -500,7 +503,7 @@
         <v>63.89</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -520,7 +523,7 @@
         <v>70.56</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -540,7 +543,7 @@
         <v>80.010000000000005</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
implimentation of parallization using testng and code update accordingly
</commit_message>
<xml_diff>
--- a/src/test/resources/bulkDataXLSX.xlsx
+++ b/src/test/resources/bulkDataXLSX.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="31">
   <si>
     <t>Subhash</t>
   </si>
@@ -109,6 +109,15 @@
   </si>
   <si>
     <t>2025-01-01 07:27:49</t>
+  </si>
+  <si>
+    <t>2025-01-03 07:31:39</t>
+  </si>
+  <si>
+    <t>2025-01-06 08:51:11</t>
+  </si>
+  <si>
+    <t>2025-01-06 08:51:12</t>
   </si>
 </sst>
 </file>
@@ -483,7 +492,7 @@
         <v>85</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -503,7 +512,7 @@
         <v>63.89</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -523,7 +532,7 @@
         <v>70.56</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -543,7 +552,7 @@
         <v>80.010000000000005</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated code for failed tests
</commit_message>
<xml_diff>
--- a/src/test/resources/bulkDataXLSX.xlsx
+++ b/src/test/resources/bulkDataXLSX.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="32">
   <si>
     <t>Subhash</t>
   </si>
@@ -118,6 +118,9 @@
   </si>
   <si>
     <t>2025-01-06 08:51:12</t>
+  </si>
+  <si>
+    <t>2025-01-12 08:26:54</t>
   </si>
 </sst>
 </file>
@@ -492,7 +495,7 @@
         <v>85</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -512,7 +515,7 @@
         <v>63.89</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -532,7 +535,7 @@
         <v>70.56</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -552,7 +555,7 @@
         <v>80.010000000000005</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>